<commit_message>
Datasheet input parameterization step update
</commit_message>
<xml_diff>
--- a/RunManager.xlsx
+++ b/RunManager.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Aishwarya\eclipse\Workspace\git_repo_projects\Maven-Java-BDDFramework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2C450C0-2A24-4035-A905-27F16F59DD9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A64DD8C-3023-49D9-9C46-01B60CCB0BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="11">
   <si>
     <t>TestCaseName</t>
   </si>
@@ -52,6 +52,12 @@
   </si>
   <si>
     <t>Pass</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Fail</t>
   </si>
 </sst>
 </file>
@@ -412,10 +418,10 @@
         <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" t="s" s="1">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -428,7 +434,7 @@
       <c r="C3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D3" t="s" s="1">
+      <c r="D3" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -440,7 +446,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>8</v>

</xml_diff>